<commit_message>
Add "设备型号" field, placed between "设备名称" and "设备是否启用"
- Removed "标签" column from device sheet
- Added "设备型号" (device_model) field to Device model
- Updated loader to recognize "设备型号" header
- Updated _resolve_template to support {设备型号} variable
- Regenerated example Excel template

Device sheet column order:
  设备分类 | 设备名称 | 设备型号 | 设备是否启用 | 带外管理IP | ...

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -443,42 +443,42 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>设备型号</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>设备是否启用</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>带外管理IP</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>设备是否启用</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>带外管理用户名</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>带外管理密码</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>带内管理IP</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>带内管理用户名</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>带内管理密码</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>标签</t>
         </is>
       </c>
     </row>
@@ -545,14 +545,11 @@
           <t>L1-示例-01</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>10.0.2.101</t>
@@ -585,14 +582,11 @@
           <t>L2-示例-01</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>10.0.3.101</t>
@@ -645,9 +639,6 @@
           <t>Admin@123</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
           <t>RM211,机柜</t>
@@ -739,7 +730,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -775,7 +765,6 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -811,7 +800,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -847,7 +835,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -883,7 +870,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -919,7 +905,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -955,7 +940,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -991,7 +975,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1027,7 +1010,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1063,7 +1045,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1099,7 +1080,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1135,7 +1115,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1171,7 +1150,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1207,7 +1185,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1243,7 +1220,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1279,7 +1255,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1315,7 +1290,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1351,7 +1325,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1387,7 +1360,6 @@
           <t>L1</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1423,7 +1395,6 @@
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1459,7 +1430,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1495,7 +1465,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1531,7 +1500,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1567,7 +1535,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1603,7 +1570,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1639,7 +1605,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1675,7 +1640,6 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1711,7 +1675,6 @@
           <t>RM211</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1747,7 +1710,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>
@@ -1783,7 +1745,6 @@
           <t>A3</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>{device_group}/{device_name}/{task_name}</t>

</xml_diff>

<commit_message>
Add device model matching to task-device filtering
Task list "标签" column replaced with "设备型号":
- match_models: comma-separated device models (AT900A3,RM211)
- Device must match ONE of the task's specified models
- Empty match_models = match all models (no filter)
- Matching order: group → model → tags

Device sheet: 标签 → 设备型号
Task sheet: 标签 → 设备型号 (comma-separated for multiple)

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -692,12 +692,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>标签</t>
+          <t>设备型号</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>截图保存目录</t>
+          <t>输出目录模板</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">

</xml_diff>

<commit_message>
fix(template): remove dead 设备型号 column from Excel template
- Both sheets (设备信息, 任务列表) had 设备型号 column from removed Device.device_model field
- 任务列表 8 cols triggered legacy parsing path instead of simplified path
- Fix demo device data to match correct column positions
- Now 任务列表 is 7 cols → simplified path, 设备信息 is 9 cols

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -443,40 +443,35 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>设备型号</t>
+          <t>设备是否启用</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>设备是否启用</t>
+          <t>带外管理IP</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>带外管理IP</t>
+          <t>带外管理用户名</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>带外管理用户名</t>
+          <t>带外管理密码</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>带外管理密码</t>
+          <t>带内管理IP</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>带内管理IP</t>
+          <t>带内管理用户名</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t>带内管理用户名</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
         <is>
           <t>带内管理密码</t>
         </is>
@@ -495,12 +490,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>192.168.1.101</t>
+          <t>是</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>192.168.1.200</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,11 +521,6 @@
       <c r="I2" t="inlineStr">
         <is>
           <t>Root@123</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>A3,计算节点</t>
         </is>
       </c>
     </row>
@@ -545,11 +535,14 @@
           <t>L1-示例-01</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>10.0.2.101</t>
@@ -563,11 +556,6 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>Admin@123</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>L1,交换机</t>
         </is>
       </c>
     </row>
@@ -582,11 +570,14 @@
           <t>L2-示例-01</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>10.0.3.101</t>
@@ -600,11 +591,6 @@
       <c r="I4" t="inlineStr">
         <is>
           <t>Admin@123</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>L2,交换机</t>
         </is>
       </c>
     </row>
@@ -621,12 +607,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>192.168.4.101</t>
+          <t>是</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>192.168.4.200</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -639,11 +625,9 @@
           <t>Admin@123</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>RM211,机柜</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -656,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -692,20 +676,15 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>设备型号</t>
+          <t>输出目录模板</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>输出目录模板</t>
+          <t>图片命名格式</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
-        <is>
-          <t>图片命名格式</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
         <is>
           <t>是否启用</t>
         </is>
@@ -730,17 +709,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -765,17 +744,17 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -800,17 +779,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -835,17 +814,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -870,17 +849,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -905,17 +884,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -940,17 +919,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -975,17 +954,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1010,17 +989,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1045,17 +1024,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1080,17 +1059,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1115,17 +1094,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1150,17 +1129,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1185,17 +1164,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1220,17 +1199,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1255,17 +1234,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1290,17 +1269,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1325,17 +1304,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1360,17 +1339,17 @@
           <t>L1</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1395,17 +1374,17 @@
           <t>L1/L2</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
         <is>
           <t>是</t>
         </is>
@@ -1430,17 +1409,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1465,17 +1444,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1500,17 +1479,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1535,17 +1514,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1570,17 +1549,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1605,17 +1584,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1640,17 +1619,17 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1675,17 +1654,17 @@
           <t>RM211</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1710,17 +1689,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
         <is>
           <t>否</t>
         </is>
@@ -1745,17 +1724,17 @@
           <t>A3</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>{device_group}/{device_name}/{task_name}</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{device_name}_{task_name}_{timestamp}</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="H31" t="inlineStr">
         <is>
           <t>否</t>
         </is>

</xml_diff>

<commit_message>
fix: log disabled devices/tasks and unmatched tasks in plan_generator
- Log disabled devices and tasks so users can see what was filtered
- Log tasks that matched zero devices (group mismatch warning)
- Remove orphaned 拔插硬盘后清除Foreign配置 from Excel template

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -540,9 +540,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>10.0.2.101</t>
@@ -575,9 +572,6 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>10.0.3.101</t>
@@ -625,9 +619,6 @@
           <t>Admin@123</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -640,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1700,41 +1691,6 @@
         </is>
       </c>
       <c r="G30" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>拔插硬盘后清除Foreign配置</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>BMC</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
         <is>
           <t>否</t>
         </is>

</xml_diff>

<commit_message>
docs: update example Excel template to bilingual headers
Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -433,47 +433,47 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>设备分类</t>
+          <t>设备分类(DeviceGroup)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>设备名称</t>
+          <t>设备名称(DeviceName)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>设备是否启用</t>
+          <t>设备是否启用(DeviceEnabled)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>带外管理IP</t>
+          <t>带外管理IP(OOB_IP)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>带外管理用户名</t>
+          <t>带外管理用户名(OOB_Username)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>带外管理密码</t>
+          <t>带外管理密码(OOB_Password)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>带内管理IP</t>
+          <t>带内管理IP(IB_IP)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>带内管理用户名</t>
+          <t>带内管理用户名(IB_Username)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>带内管理密码</t>
+          <t>带内管理密码(IB_Password)</t>
         </is>
       </c>
     </row>
@@ -647,37 +647,37 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>任务序号</t>
+          <t>任务序号(TaskSequence)</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>任务名称</t>
+          <t>任务名称(TaskName)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>任务类型</t>
+          <t>任务类型(TaskType)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>设备分组</t>
+          <t>设备分组(DeviceGroup)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>输出目录模板</t>
+          <t>截图保存目录(OutputDir)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>图片命名格式</t>
+          <t>图片命名格式(FileNamePattern)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>是否启用</t>
+          <t>是否启用(Enabled)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: CI assets packaging + MHTML empty data guard + template defaults
CI:
- Add assets/ to app layer and full release assembly (SVGs were missing from package)

MHTML:
- Check for empty data before writing file
- Log distinct warning when CDP returns empty MHTML data

Template:
- Add {TaskIP} smart variable: BMC→OOB_IP, SSH→IB_IP
- Update example Excel default OutputDir/FileNamePattern

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -702,12 +702,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -737,12 +737,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -772,12 +772,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -807,12 +807,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -842,12 +842,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -877,12 +877,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -947,12 +947,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -982,12 +982,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1017,12 +1017,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1052,12 +1052,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1087,12 +1087,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1157,12 +1157,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1192,12 +1192,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1227,12 +1227,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1297,12 +1297,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1367,12 +1367,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1402,12 +1402,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1472,12 +1472,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1507,12 +1507,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1542,12 +1542,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1577,12 +1577,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1612,12 +1612,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1647,12 +1647,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1682,12 +1682,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>{device_group}/{device_name}/{task_name}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>{device_name}_{task_name}_{timestamp}</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">

</xml_diff>

<commit_message>
fix: evidence.html as real DOM + addressbar via set_content + FullScreenshot field
evidence.html:
- Save rendered DOM (document.documentElement.outerHTML) instead of embedded PNG
- Remove script tags and event handlers for offline safety
- Preserves all DOM elements: buttons, tables, inputs, text content

Address bar:
- Use page.set_content() to load SVG inline (avoids file:// security block)
- Reuse existing browser context instead of launching separate browser
- logger.exception() for diagnostics when compose fails

FullScreenshot + ScreenshotMode:
- New Task fields: full_screenshot (bool), screenshot_mode (str)
- Excel headers: 是否全量截图(FullScreenshot), 截图模式(ScreenshotMode)
- SSH: PNG truncated to 100 lines when FullScreenshot=false
- BMC: content-aware screenshot with scroll container detection + blank crop

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -680,6 +680,16 @@
           <t>是否启用(Enabled)</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>是否全量截图(FullScreenshot)</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>截图模式(ScreenshotMode)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -715,6 +725,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -750,6 +770,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -785,6 +815,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -820,6 +860,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -855,6 +905,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -890,6 +950,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -925,6 +995,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -960,6 +1040,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -995,6 +1085,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1030,6 +1130,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1065,6 +1175,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1100,6 +1220,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1135,6 +1265,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1170,6 +1310,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1205,6 +1355,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1240,6 +1400,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1275,6 +1445,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1310,6 +1490,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1345,6 +1535,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1380,6 +1580,16 @@
           <t>是</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1415,6 +1625,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1450,6 +1670,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1485,6 +1715,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1520,6 +1760,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1555,6 +1805,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1590,6 +1850,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1625,6 +1895,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1660,6 +1940,16 @@
           <t>否</t>
         </is>
       </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>auto</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1693,6 +1983,16 @@
       <c r="G30" t="inlineStr">
         <is>
           <t>否</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>auto</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: unify plan task identity and checks
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -631,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -647,982 +647,1087 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>任务ID(TaskID)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>任务序号(TaskSequence)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>任务名称(TaskName)</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>任务类型(TaskType)</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>设备分组(DeviceGroup)</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>截图保存目录(OutputDir)</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>图片命名格式(FileNamePattern)</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>是否启用(Enabled)</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>是否全量截图(FullScreenshot)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>截图模式(ScreenshotMode)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>task.001</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>RAID配置测试</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>task.002</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>机柜RM211的管理iBMC IP查询和设置测试</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>RM211</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>task.003</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>计算节点远程上电和下电测试</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>task.004</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-资产摘要</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>task.005</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-网络适配器</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>task.006</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-门限传感器</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>task.007</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-电源信息</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>task.008</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-风扇信息</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>task.009</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>风扇冗余测试</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>task.010</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>A3 BMC首页截图</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>task.011</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>操作系统安装测试</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>task.012</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>NPU驱动和固件安装测试</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>task.013</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>灵衢网络管理网口IP查询和设置测试</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>task.014</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>计算节点电子标签查询测试</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>task.015</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>计算节点灵衢总线板与灵衢总线和以太板CPLD版本信息查询测试</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>task.016</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>计算节点光口状态查询测试</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>task.017</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>计算节点光模块信息查询测试</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>L1/L2/A3</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>task.018</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>计算节点温度管理测试</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>task.019</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>计算节点L1交换网络端口查询测试</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>L1</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>task.020</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>模块拔插告警上报测试</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>SSH</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>L1/L2</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>是</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>task.021</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>计算节点上电测试-内存</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1632,42 +1737,47 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>task.022</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>计算节点上电测试-CPU</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1677,42 +1787,47 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>task.023</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
         <v>23</v>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>计算节点iBMC IP查询和设置测试</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1722,42 +1837,47 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>task.024</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
         <v>24</v>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-CPU</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1767,42 +1887,47 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>task.025</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
         <v>25</v>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-NPU</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1812,42 +1937,47 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>task.026</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
         <v>26</v>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>计算节点部件信息查询测试-内存</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1857,42 +1987,47 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>task.027</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
         <v>27</v>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>电源冗余测试</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>RM211</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1902,42 +2037,47 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>task.028</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
         <v>28</v>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>硬盘冗余测试-系统日志</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>RM211</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1947,42 +2087,47 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
           <t>auto</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>task.029</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
         <v>29</v>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>硬盘冗余测试</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>BMC</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>A3</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
-        </is>
-      </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>{TaskIP}_{TaskName}_{timestamp}</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1991,6 +2136,11 @@
         </is>
       </c>
       <c r="I30" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
         <is>
           <t>auto</t>
         </is>
@@ -2016,7 +2166,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>任务配置分为两层：</t>
+          <t>任务配置分为两层：Excel 任务列表使用任务ID(TaskID)作为稳定主键，tasks.json 以相同任务ID作为 key；任务名称仅用于展示。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add acceptance docx export
</commit_message>
<xml_diff>
--- a/examples/task_template.xlsx
+++ b/examples/task_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="设备信息" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="任务列表" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="说明" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备信息" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务列表" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -634,12 +634,12 @@
   <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
@@ -692,8 +692,10 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>4.1.8</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -712,12 +714,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -737,8 +739,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4.2.1</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -757,12 +761,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -782,8 +786,10 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>4.2.3</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -802,12 +808,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -827,8 +833,10 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -847,12 +855,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -872,8 +880,10 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -892,12 +902,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -917,8 +927,10 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -937,12 +949,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -962,8 +974,10 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -982,12 +996,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1007,8 +1021,10 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1027,12 +1043,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1052,8 +1068,10 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>9</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>4.3.3</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1072,12 +1090,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1097,8 +1115,10 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>10</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1117,12 +1137,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -1142,8 +1162,10 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>11</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>4.1.9</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1162,12 +1184,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1187,8 +1209,10 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>12</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>4.1.10</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1207,12 +1231,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1232,8 +1256,10 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>13</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4.1.11</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -1252,12 +1278,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1277,8 +1303,10 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>14</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>4.1.12</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -1297,12 +1325,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1322,8 +1350,10 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4.1.13</t>
+        </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -1342,12 +1372,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1367,8 +1397,10 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4.1.14</t>
+        </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -1387,12 +1419,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1412,8 +1444,10 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>4.1.15</t>
+        </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -1432,12 +1466,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1457,8 +1491,10 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>4.1.16</t>
+        </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -1477,12 +1513,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1502,8 +1538,10 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>19</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>4.2.5</t>
+        </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -1522,12 +1560,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1547,8 +1585,10 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>20</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>4.3.5</t>
+        </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -1567,12 +1607,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1592,8 +1632,10 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>4.1.7</t>
+        </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -1612,12 +1654,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1637,8 +1679,10 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>4.1.7</t>
+        </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -1657,12 +1701,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1682,8 +1726,10 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>4.2.2</t>
+        </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -1702,12 +1748,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1727,8 +1773,10 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -1747,12 +1795,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1772,8 +1820,10 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -1792,12 +1842,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1817,8 +1867,10 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>4.2.4</t>
+        </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -1837,12 +1889,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1862,8 +1914,10 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>4.3.2</t>
+        </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1882,12 +1936,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1907,8 +1961,10 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>4.3.4</t>
+        </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -1927,12 +1983,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1952,8 +2008,10 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>4.3.4</t>
+        </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1972,12 +2030,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>{TaskSequence}_{TaskName}/{DeviceGroup}</t>
+          <t>{任务序号}.{任务名称}/{设备分类}</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>{TaskIP}_{TaskName}_{timestamp}</t>
+          <t>{TaskIP}-{任务名称}</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2007,7 +2065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2023,21 +2081,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>1. Excel 任务列表 — 只配置匹配信息：序号/名称/类型/分组/标签/输出目录/命名格式/启用</t>
+          <t>1. Excel 任务列表 — 配置文档用例编号/名称/类型/分组/输出目录/命名格式/启用；任务序号应与验收文档用例编号一致。</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. tasks.json — 执行细节：URL/命令/超时/重试/规则，通过任务名称匹配</t>
+          <t>2. 默认截图目录：{任务序号}.{任务名称}/{设备分类}；默认截图名：{TaskIP}-{任务名称}。</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Agent 可远程推送更新 tasks.json，无需修改 Excel</t>
+          <t>3. tasks.json — 执行细节：URL/命令/超时/重试/规则，通过任务名称匹配。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. 任务名称带“-子场景”的任务会回填到同名父用例的测试结果框。</t>
         </is>
       </c>
     </row>

</xml_diff>